<commit_message>
Update SandLock owner dashboard and reservation backend
</commit_message>
<xml_diff>
--- a/data/SandLock_Dashboard_Database.xlsx
+++ b/data/SandLock_Dashboard_Database.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Users" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reservations" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access Logs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device Events" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alerts" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feedback" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lockers" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Audit" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Users" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Reservations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Access Logs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Device Events" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Alerts" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Payments" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Feedback" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Lockers" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Admin Audit" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,6 +569,128 @@
       <c r="S1" t="inlineStr">
         <is>
           <t>Cancelled At</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>User ID</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Updated At</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Revision</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Financial Outcome</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SL-4322bc50-0f2b-4c21-a4e2-01977cea1417</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>01143873330</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>mayar elhady</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>22:22</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>23:22</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-09-22T22:22:00.000Z</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-09-22T23:22:00.000Z</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>[REDACTED]</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L2" t="n">
+        <v>20</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>20</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>demo-only</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>2026-09-22T22:21:31.928Z</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>2026-09-22T22:22:36.588Z</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>usr_3aec4bc0b8ace08e981cfc0b7b852abe</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>2026-09-22T22:22:36.588Z</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>3</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>demo-final</t>
         </is>
       </c>
     </row>
@@ -736,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -773,6 +895,75 @@
       <c r="G1" t="inlineStr">
         <is>
           <t>Reference</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Financial Event</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Financial Outcome</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Final Demo Value</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Actual Collected Revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-22T22:21:31.928Z</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SL-4322bc50-0f2b-4c21-a4e2-01977cea1417</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Demo Booking Value</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>demo-only</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PAY-SL-4322bc50-0f2b-4c21-a4e2-01977cea1417</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>PAY-SL-4322bc50-0f2b-4c21-a4e2-01977cea1417</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>demo-final</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -828,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -875,6 +1066,78 @@
       <c r="I1" t="inlineStr">
         <is>
           <t>Current Booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>reserved</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>occupied</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>offline</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>offline</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update SandLock control backend and dashboard
</commit_message>
<xml_diff>
--- a/data/SandLock_Dashboard_Database.xlsx
+++ b/data/SandLock_Dashboard_Database.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -689,6 +689,414 @@
         <v>3</v>
       </c>
       <c r="W2" t="inlineStr">
+        <is>
+          <t>demo-final</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SL-5ef2a238-8c6c-4daa-b7c0-0da6c78d6146</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>01143873330</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>mayar elhady</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>23 Sep 2026</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>09:13 PM</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>10:13 PM</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:13:00.000Z</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-09-23T19:13:00.000Z</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>[REDACTED]</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>20</v>
+      </c>
+      <c r="L3" t="n">
+        <v>20</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>20</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Cancelled</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>demo-only</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:12:44.784Z</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:30:53.713Z</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>usr_e0c4352339bc2ff7ff8c5cd068c831e3</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:30:53.713Z</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>3</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>demo-final</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SL-4b19d0b8-0cf5-4b36-ae8d-d9ce1e667517</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>01143873330</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>mayar elhady</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>23 Sep 2026</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>09:32 PM</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>10:32 PM</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:32:00.000Z</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-09-23T19:32:00.000Z</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>[REDACTED]</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>20</v>
+      </c>
+      <c r="L4" t="n">
+        <v>20</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>20</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Cancelled</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>demo-only</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:31:13.123Z</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:32:36.098Z</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>usr_e0c4352339bc2ff7ff8c5cd068c831e3</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:32:36.098Z</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>3</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>demo-final</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SL-825ca2c5-ea12-4147-b513-c62d32ded2cd</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>01143873330</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>mayar elhady</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>23 Sep 2026</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>09:34 PM</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>10:35 PM</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:34:00.000Z</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-09-23T19:35:00.000Z</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>[REDACTED]</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>20</v>
+      </c>
+      <c r="L5" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>demo-only</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:34:30.874Z</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:34:46.362Z</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>usr_e0c4352339bc2ff7ff8c5cd068c831e3</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:34:46.362Z</t>
+        </is>
+      </c>
+      <c r="V5" t="n">
+        <v>2</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>demo-final</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SL-fa0fb203-ec66-4056-8d5a-6157dbc2f733</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>01143873330</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>mayar elhady</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>23 Sep 2026</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>09:35 PM</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>10:35 PM</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:35:00.000Z</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-09-23T19:35:00.000Z</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>[REDACTED]</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>18</v>
+      </c>
+      <c r="L6" t="n">
+        <v>18</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>18</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>demo-only</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:35:08.589Z</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:35:16.627Z</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>usr_e0c4352339bc2ff7ff8c5cd068c831e3</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:35:16.627Z</t>
+        </is>
+      </c>
+      <c r="V6" t="n">
+        <v>2</v>
+      </c>
+      <c r="W6" t="inlineStr">
         <is>
           <t>demo-final</t>
         </is>
@@ -858,7 +1266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -929,7 +1337,6 @@
           <t>SL-4322bc50-0f2b-4c21-a4e2-01977cea1417</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>Demo Booking Value</t>
@@ -962,6 +1369,199 @@
         <v>20</v>
       </c>
       <c r="K2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:12:44.784Z</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SL-5ef2a238-8c6c-4daa-b7c0-0da6c78d6146</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Demo Booking Value</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>demo-only</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PAY-SL-5ef2a238-8c6c-4daa-b7c0-0da6c78d6146</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>PAY-SL-5ef2a238-8c6c-4daa-b7c0-0da6c78d6146</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>demo-final</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>20</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:31:13.123Z</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SL-4b19d0b8-0cf5-4b36-ae8d-d9ce1e667517</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Demo Booking Value</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>demo-only</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PAY-SL-4b19d0b8-0cf5-4b36-ae8d-d9ce1e667517</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>PAY-SL-4b19d0b8-0cf5-4b36-ae8d-d9ce1e667517</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>demo-final</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>20</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:34:30.874Z</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SL-825ca2c5-ea12-4147-b513-c62d32ded2cd</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Demo Booking Value</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>demo-only</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PAY-SL-825ca2c5-ea12-4147-b513-c62d32ded2cd</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>PAY-SL-825ca2c5-ea12-4147-b513-c62d32ded2cd</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>demo-final</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-23T18:35:08.589Z</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SL-fa0fb203-ec66-4056-8d5a-6157dbc2f733</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Demo Booking Value</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>18</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>demo-only</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PAY-SL-fa0fb203-ec66-4056-8d5a-6157dbc2f733</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>PAY-SL-fa0fb203-ec66-4056-8d5a-6157dbc2f733</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>demo-final</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>